<commit_message>
Correct Globus exclusion reason to non-consolidated holding statements
</commit_message>
<xml_diff>
--- a/2026 New/Results_severe_P1_decline_analysis.xlsx
+++ b/2026 New/Results_severe_P1_decline_analysis.xlsx
@@ -185,7 +185,7 @@
     <t>Zakłady Mięsne Henryk Kania SA w upadłości | NIP 7440003325 | Removed from analysis | firms=1, rows=1 | Reason [LIQUIDATION]: Non-comparable financial statements due to liquidation.</t>
   </si>
   <si>
-    <t>Globus sp. z o.o., Warszawa | NIP 7773261746 | Removed from analysis | firms=1, rows=1 | Reason [EXTREME_PROFITABILITY_RATIO]: Extreme net-profit/sales ratio from a very small sales denominator; dominates profitability variation in regression analysis.</t>
+    <t>Globus sp. z o.o., Warszawa | NIP 7773261746 | Removed from analysis | firms=1, rows=1 | Reason [HOLDING_NONCONSOLIDATED]: Non-comparable financial statements: holding company reports non-consolidated financial statements.</t>
   </si>
   <si>
     <t>RANK2019 (primary) and RANK2019_MANUFACTURING (secondary). Internal shared masks are Rank2019 and Rank2019_Manufacturing. Manufacturing is nested within ranking; these are not independent replications.</t>
@@ -2136,7 +2136,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="15" spans="1:2" ht="60" customHeight="1">
+    <row r="15" spans="1:2" ht="46" customHeight="1">
       <c r="A15" s="6" t="s">
         <v>13</v>
       </c>

</xml_diff>

<commit_message>
Move supplementary manual exclusions to the end of regression READMEs
</commit_message>
<xml_diff>
--- a/2026 New/Results_severe_P1_decline_analysis.xlsx
+++ b/2026 New/Results_severe_P1_decline_analysis.xlsx
@@ -47,6 +47,102 @@
     <t>Output file</t>
   </si>
   <si>
+    <t>Samples</t>
+  </si>
+  <si>
+    <t>Price basis</t>
+  </si>
+  <si>
+    <t>Primary definition</t>
+  </si>
+  <si>
+    <t>Robustness</t>
+  </si>
+  <si>
+    <t>Sample and missingness</t>
+  </si>
+  <si>
+    <t>Group profile</t>
+  </si>
+  <si>
+    <t>Logit outcome</t>
+  </si>
+  <si>
+    <t>Logit predictors</t>
+  </si>
+  <si>
+    <t>Timing</t>
+  </si>
+  <si>
+    <t>Logit estimator</t>
+  </si>
+  <si>
+    <t>Logit inference</t>
+  </si>
+  <si>
+    <t>Model statistics</t>
+  </si>
+  <si>
+    <t>AIC/BIC</t>
+  </si>
+  <si>
+    <t>Average marginal effects</t>
+  </si>
+  <si>
+    <t>P2 outcome</t>
+  </si>
+  <si>
+    <t>P3 outcome</t>
+  </si>
+  <si>
+    <t>Growth preprocessing</t>
+  </si>
+  <si>
+    <t>Growth controls</t>
+  </si>
+  <si>
+    <t>Selected interaction</t>
+  </si>
+  <si>
+    <t>Interaction audit</t>
+  </si>
+  <si>
+    <t>Influence warning</t>
+  </si>
+  <si>
+    <t>Raw-growth mean warning</t>
+  </si>
+  <si>
+    <t>P2 lag sensitivity</t>
+  </si>
+  <si>
+    <t>Estimator comparison</t>
+  </si>
+  <si>
+    <t>Firth implementation</t>
+  </si>
+  <si>
+    <t>FULL</t>
+  </si>
+  <si>
+    <t>Quantile distinction</t>
+  </si>
+  <si>
+    <t>Interpretation cautions</t>
+  </si>
+  <si>
+    <t>Model status</t>
+  </si>
+  <si>
+    <t>Method source</t>
+  </si>
+  <si>
+    <t>Penalised LR reference</t>
+  </si>
+  <si>
+    <t>Reproduce</t>
+  </si>
+  <si>
     <t>Manual exclusions</t>
   </si>
   <si>
@@ -68,102 +164,6 @@
     <t>Manual exclusion 6</t>
   </si>
   <si>
-    <t>Samples</t>
-  </si>
-  <si>
-    <t>Price basis</t>
-  </si>
-  <si>
-    <t>Primary definition</t>
-  </si>
-  <si>
-    <t>Robustness</t>
-  </si>
-  <si>
-    <t>Sample and missingness</t>
-  </si>
-  <si>
-    <t>Group profile</t>
-  </si>
-  <si>
-    <t>Logit outcome</t>
-  </si>
-  <si>
-    <t>Logit predictors</t>
-  </si>
-  <si>
-    <t>Timing</t>
-  </si>
-  <si>
-    <t>Logit estimator</t>
-  </si>
-  <si>
-    <t>Logit inference</t>
-  </si>
-  <si>
-    <t>Model statistics</t>
-  </si>
-  <si>
-    <t>AIC/BIC</t>
-  </si>
-  <si>
-    <t>Average marginal effects</t>
-  </si>
-  <si>
-    <t>P2 outcome</t>
-  </si>
-  <si>
-    <t>P3 outcome</t>
-  </si>
-  <si>
-    <t>Growth preprocessing</t>
-  </si>
-  <si>
-    <t>Growth controls</t>
-  </si>
-  <si>
-    <t>Selected interaction</t>
-  </si>
-  <si>
-    <t>Interaction audit</t>
-  </si>
-  <si>
-    <t>Influence warning</t>
-  </si>
-  <si>
-    <t>Raw-growth mean warning</t>
-  </si>
-  <si>
-    <t>P2 lag sensitivity</t>
-  </si>
-  <si>
-    <t>Estimator comparison</t>
-  </si>
-  <si>
-    <t>Firth implementation</t>
-  </si>
-  <si>
-    <t>FULL</t>
-  </si>
-  <si>
-    <t>Quantile distinction</t>
-  </si>
-  <si>
-    <t>Interpretation cautions</t>
-  </si>
-  <si>
-    <t>Model status</t>
-  </si>
-  <si>
-    <t>Method source</t>
-  </si>
-  <si>
-    <t>Penalised LR reference</t>
-  </si>
-  <si>
-    <t>Reproduce</t>
-  </si>
-  <si>
     <t>Supplementary P1 vulnerability → P2 recovery → P3 subsequent development analysis. Associations are descriptive, not causal.</t>
   </si>
   <si>
@@ -173,6 +173,102 @@
     <t>Results_severe_P1_decline_analysis.xlsx</t>
   </si>
   <si>
+    <t>RANK2019 (primary) and RANK2019_MANUFACTURING (secondary). Internal shared masks are Rank2019 and Rank2019_Manufacturing. Manufacturing is nested within ranking; these are not independent replications.</t>
+  </si>
+  <si>
+    <t>Nominal sales growth. All model outcomes and lags follow code_config.PERIOD_MODEL_SETTINGS.</t>
+  </si>
+  <si>
+    <t>BottomP1_20 = 1 only when ngrowth_P1 &lt; -0.20; equality is outside the severe group. Membership is fixed by P1.</t>
+  </si>
+  <si>
+    <t>Repeat the logit, P2/P3 group models, and profitability interactions separately at -15%, -20%, -25%. Never include multiple threshold indicators in one model.</t>
+  </si>
+  <si>
+    <t>Apply the same ranking/manufacturing and complete-trajectory masks as main OLS, then the same period-specific complete-case exclusions. Missing P1 growth has unknown membership, never zero.</t>
+  </si>
+  <si>
+    <t>Raw simple P1/P2/P3 growth and 2019 starting covariates; N, mean, median, sample SD. Profile shares use the selected complete-trajectory sample, not the smaller regression samples.</t>
+  </si>
+  <si>
+    <t>BottomP1_20 (0/1), neither standardised nor winsorised. P1=2019-2020 simple growth determines membership; log-growth columns are not compared with percentage thresholds.</t>
+  </si>
+  <si>
+    <t>ln_sales_start_P1, profit_margin_start_P1, export_ratio_start_P1, asset_turnover_start_P1, capital_ratio_start_P1, sales_per_employee_start_P1, owner_num, export_ratio_x_ln_sales_start_P1, lag_ngrowth_log_ann_P1; sector controls.</t>
+  </si>
+  <si>
+    <t>P1 start covariates are from 2019; P1 lag is 2018-2019. No P1 realised outcome, P2/P3 predictor or trajectory label enters the logit. Ownership/sector use the established stable descriptors, treated as predetermined.</t>
+  </si>
+  <si>
+    <t>Firth bias-reduced logistic regression for both selected samples and all thresholds; full firm samples and sector controls retained. Manufacturing health/pharma has zero severe cases at all thresholds.</t>
+  </si>
+  <si>
+    <t>Wald coefficient z tests and 95% intervals using inverse expected Fisher information; odds-ratio intervals exponentiate coefficient intervals. They are not profile-penalised intervals.</t>
+  </si>
+  <si>
+    <t>McFadden pseudo-R² uses unpenalised log-likelihood at the fitted coefficients versus intercept-only ML. LR is penalised for Firth and constrains all slopes to zero using the same full-design Jeffreys penalty.</t>
+  </si>
+  <si>
+    <t>AIC_plug_in and BIC_plug_in evaluate the unpenalised likelihood at bias-reduced estimates. They are descriptive, not conventional MLE model-selection criteria. Do not compare them across thresholds with different responses.</t>
+  </si>
+  <si>
+    <t>Preferred probability-scale interpretation. Continuous AMEs are average total derivatives per one SD, including the chain rule for export_ratio × ln_sales. Binary ownership and sector effects are average discrete probability differences; delta-method Wald intervals.</t>
+  </si>
+  <si>
+    <t>Nominal annualised log sales growth (2020-2022); (ln(sales_2022) - ln(sales_2020)) / 2</t>
+  </si>
+  <si>
+    <t>Nominal annualised log sales growth (2022-2024); (ln(sales_2024) - ln(sales_2022)) / 2</t>
+  </si>
+  <si>
+    <t>Use principal OLS winsor_std: clip only the outcome at 1%/99%, then standardise it and metadata-designated continuous predictors within the same period estimation sample (ddof=0). Group indicators remain 0/1.</t>
+  </si>
+  <si>
+    <t>Same period starting covariates, ownership, export_ratio × ln_sales, sector controls and lag growth as main OLS. P2's group coefficient is conditional on P1 growth through its lag; it is an incremental threshold association.</t>
+  </si>
+  <si>
+    <t>Only standardised profit_margin × BottomP1, estimated separately for P2 and P3. Do not restandardise this product. The ordinary-firm slope is β1, the severe-group slope β1+β3, and the slope difference β3. The group main effect is evaluated at mean profitability.</t>
+  </si>
+  <si>
+    <t>Both profitability main effect and interaction use exactly the same z-score; combined inference uses Var(β1)+Var(β3)+2Cov(β1,β3). No scaling mismatch was found.</t>
+  </si>
+  <si>
+    <t>The manual-exclusion audit at the end of this README records earlier influential firms and their comparability reasons. Recomputed VIF, subgroup-variation and influence diagnostics describe the current samples. Remaining influential observations can still affect inference; these exclusions alone do not establish robustness.</t>
+  </si>
+  <si>
+    <t>Descriptive growth is raw and can be affected by extreme observations. Compare means with the appended medians, 5th/95th percentiles, maxima and mean-without-largest diagnostics.</t>
+  </si>
+  <si>
+    <t>An additional -20% diagnostic removes the continuous P1-growth lag on exactly the same sample and outcome scaling. It does not replace the primary model. Both versions remain conditional associations, not causal recovery effects.</t>
+  </si>
+  <si>
+    <t>Ordinary MLE works without separation for Rank2019 at all thresholds. Firth was deliberately used in both samples for consistency and is retained. The principal ranking MLE comparison is diagnostic only; manufacturing requires separation handling.</t>
+  </si>
+  <si>
+    <t>Project-local NumPy/SciPy adjusted-score solver, not execution of the R logistf package. Coefficients independently reproduced by BFGS; covariance is inverse original expected Fisher information. Wald/delta intervals are approximate, particularly for sparse or separated cells.</t>
+  </si>
+  <si>
+    <t>No FULL model: group definition mechanically contains part of FULL growth.</t>
+  </si>
+  <si>
+    <t>Fixed realised-P1 firm groups followed over time; no conditional-quantile models are estimated.</t>
+  </si>
+  <si>
+    <t>Complete-trajectory selection excludes firms without later outcomes. Subsequent covariates and lags may mediate earlier decline; group comparisons and interactions are conditional associations, not causal recovery effects. Firth reduces first-order coefficient bias; it does not guarantee every fitted probability moves toward one half.</t>
+  </si>
+  <si>
+    <t>6 logistic, 12 group OLS, 12 interaction OLS primary/threshold models completed. 0 explicitly flagged failures. Audit diagnostics additionally compare one ranking MLE fit and two P2 fits without lag growth.</t>
+  </si>
+  <si>
+    <t>https://search.r-project.org/CRAN/refmans/logistf/html/logistf.html</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/cran/logistf/master/R/logistftest.R</t>
+  </si>
+  <si>
+    <t>python3 code_severe_p1_decline.py; shared settings remain in code_config.py. Canonical datasets and other workbooks are not modified.</t>
+  </si>
+  <si>
     <t>Enabled=True. Shared code_config.MANUAL_EXCLUSIONS; match verified NIP or exact company name (outer whitespace ignored). Applied before analytical filtering and all transformations. Canonical data retained.</t>
   </si>
   <si>
@@ -192,102 +288,6 @@
   </si>
   <si>
     <t>Ordipol sp. z o.o. (w upadłości), Bielany Wrocławskie | NIP 6772001669 | Removed from analysis | firms=1, rows=1 | Reason [LIQUIDATION]: Non-comparable financial statements due to liquidation.</t>
-  </si>
-  <si>
-    <t>RANK2019 (primary) and RANK2019_MANUFACTURING (secondary). Internal shared masks are Rank2019 and Rank2019_Manufacturing. Manufacturing is nested within ranking; these are not independent replications.</t>
-  </si>
-  <si>
-    <t>Nominal sales growth. All model outcomes and lags follow code_config.PERIOD_MODEL_SETTINGS.</t>
-  </si>
-  <si>
-    <t>BottomP1_20 = 1 only when ngrowth_P1 &lt; -0.20; equality is outside the severe group. Membership is fixed by P1.</t>
-  </si>
-  <si>
-    <t>Repeat the logit, P2/P3 group models, and profitability interactions separately at -15%, -20%, -25%. Never include multiple threshold indicators in one model.</t>
-  </si>
-  <si>
-    <t>Apply the same ranking/manufacturing and complete-trajectory masks as main OLS, then the same period-specific complete-case exclusions. Missing P1 growth has unknown membership, never zero.</t>
-  </si>
-  <si>
-    <t>Raw simple P1/P2/P3 growth and 2019 starting covariates; N, mean, median, sample SD. Profile shares use the selected complete-trajectory sample, not the smaller regression samples.</t>
-  </si>
-  <si>
-    <t>BottomP1_20 (0/1), neither standardised nor winsorised. P1=2019-2020 simple growth determines membership; log-growth columns are not compared with percentage thresholds.</t>
-  </si>
-  <si>
-    <t>ln_sales_start_P1, profit_margin_start_P1, export_ratio_start_P1, asset_turnover_start_P1, capital_ratio_start_P1, sales_per_employee_start_P1, owner_num, export_ratio_x_ln_sales_start_P1, lag_ngrowth_log_ann_P1; sector controls.</t>
-  </si>
-  <si>
-    <t>P1 start covariates are from 2019; P1 lag is 2018-2019. No P1 realised outcome, P2/P3 predictor or trajectory label enters the logit. Ownership/sector use the established stable descriptors, treated as predetermined.</t>
-  </si>
-  <si>
-    <t>Firth bias-reduced logistic regression for both selected samples and all thresholds; full firm samples and sector controls retained. Manufacturing health/pharma has zero severe cases at all thresholds.</t>
-  </si>
-  <si>
-    <t>Wald coefficient z tests and 95% intervals using inverse expected Fisher information; odds-ratio intervals exponentiate coefficient intervals. They are not profile-penalised intervals.</t>
-  </si>
-  <si>
-    <t>McFadden pseudo-R² uses unpenalised log-likelihood at the fitted coefficients versus intercept-only ML. LR is penalised for Firth and constrains all slopes to zero using the same full-design Jeffreys penalty.</t>
-  </si>
-  <si>
-    <t>AIC_plug_in and BIC_plug_in evaluate the unpenalised likelihood at bias-reduced estimates. They are descriptive, not conventional MLE model-selection criteria. Do not compare them across thresholds with different responses.</t>
-  </si>
-  <si>
-    <t>Preferred probability-scale interpretation. Continuous AMEs are average total derivatives per one SD, including the chain rule for export_ratio × ln_sales. Binary ownership and sector effects are average discrete probability differences; delta-method Wald intervals.</t>
-  </si>
-  <si>
-    <t>Nominal annualised log sales growth (2020-2022); (ln(sales_2022) - ln(sales_2020)) / 2</t>
-  </si>
-  <si>
-    <t>Nominal annualised log sales growth (2022-2024); (ln(sales_2024) - ln(sales_2022)) / 2</t>
-  </si>
-  <si>
-    <t>Use principal OLS winsor_std: clip only the outcome at 1%/99%, then standardise it and metadata-designated continuous predictors within the same period estimation sample (ddof=0). Group indicators remain 0/1.</t>
-  </si>
-  <si>
-    <t>Same period starting covariates, ownership, export_ratio × ln_sales, sector controls and lag growth as main OLS. P2's group coefficient is conditional on P1 growth through its lag; it is an incremental threshold association.</t>
-  </si>
-  <si>
-    <t>Only standardised profit_margin × BottomP1, estimated separately for P2 and P3. Do not restandardise this product. The ordinary-firm slope is β1, the severe-group slope β1+β3, and the slope difference β3. The group main effect is evaluated at mean profitability.</t>
-  </si>
-  <si>
-    <t>Both profitability main effect and interaction use exactly the same z-score; combined inference uses Var(β1)+Var(β3)+2Cov(β1,β3). No scaling mismatch was found.</t>
-  </si>
-  <si>
-    <t>The manual-exclusion audit above records earlier influential firms and their comparability reasons. Recomputed VIF, subgroup-variation and influence diagnostics describe the current samples. Remaining influential observations can still affect inference; these exclusions alone do not establish robustness.</t>
-  </si>
-  <si>
-    <t>Descriptive growth is raw and can be affected by extreme observations. Compare means with the appended medians, 5th/95th percentiles, maxima and mean-without-largest diagnostics.</t>
-  </si>
-  <si>
-    <t>An additional -20% diagnostic removes the continuous P1-growth lag on exactly the same sample and outcome scaling. It does not replace the primary model. Both versions remain conditional associations, not causal recovery effects.</t>
-  </si>
-  <si>
-    <t>Ordinary MLE works without separation for Rank2019 at all thresholds. Firth was deliberately used in both samples for consistency and is retained. The principal ranking MLE comparison is diagnostic only; manufacturing requires separation handling.</t>
-  </si>
-  <si>
-    <t>Project-local NumPy/SciPy adjusted-score solver, not execution of the R logistf package. Coefficients independently reproduced by BFGS; covariance is inverse original expected Fisher information. Wald/delta intervals are approximate, particularly for sparse or separated cells.</t>
-  </si>
-  <si>
-    <t>No FULL model: group definition mechanically contains part of FULL growth.</t>
-  </si>
-  <si>
-    <t>Fixed realised-P1 firm groups followed over time; no conditional-quantile models are estimated.</t>
-  </si>
-  <si>
-    <t>Complete-trajectory selection excludes firms without later outcomes. Subsequent covariates and lags may mediate earlier decline; group comparisons and interactions are conditional associations, not causal recovery effects. Firth reduces first-order coefficient bias; it does not guarantee every fitted probability moves toward one half.</t>
-  </si>
-  <si>
-    <t>6 logistic, 12 group OLS, 12 interaction OLS primary/threshold models completed. 0 explicitly flagged failures. Audit diagnostics additionally compare one ranking MLE fit and two P2 fits without lag growth.</t>
-  </si>
-  <si>
-    <t>https://search.r-project.org/CRAN/refmans/logistf/html/logistf.html</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/cran/logistf/master/R/logistftest.R</t>
-  </si>
-  <si>
-    <t>python3 code_severe_p1_decline.py; shared settings remain in code_config.py. Canonical datasets and other workbooks are not modified.</t>
   </si>
   <si>
     <t>Group Profile</t>
@@ -2118,7 +2118,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="12" spans="1:2" ht="60" customHeight="1">
+    <row r="12" spans="1:2" ht="32" customHeight="1">
       <c r="A12" s="6" t="s">
         <v>10</v>
       </c>
@@ -2126,7 +2126,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="13" spans="1:2" ht="46" customHeight="1">
+    <row r="13" spans="1:2" ht="32" customHeight="1">
       <c r="A13" s="6" t="s">
         <v>11</v>
       </c>
@@ -2158,7 +2158,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="46" customHeight="1">
+    <row r="17" spans="1:2" ht="60" customHeight="1">
       <c r="A17" s="6" t="s">
         <v>15</v>
       </c>
@@ -2166,7 +2166,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="18" spans="1:2" ht="32" customHeight="1">
+    <row r="18" spans="1:2" ht="46" customHeight="1">
       <c r="A18" s="6" t="s">
         <v>16</v>
       </c>
@@ -2174,7 +2174,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="19" spans="1:2" ht="32" customHeight="1">
+    <row r="19" spans="1:2" ht="46" customHeight="1">
       <c r="A19" s="6" t="s">
         <v>17</v>
       </c>
@@ -2182,7 +2182,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="20" spans="1:2" ht="32" customHeight="1">
+    <row r="20" spans="1:2" ht="46" customHeight="1">
       <c r="A20" s="6" t="s">
         <v>18</v>
       </c>
@@ -2206,7 +2206,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="23" spans="1:2" ht="46" customHeight="1">
+    <row r="23" spans="1:2" ht="60" customHeight="1">
       <c r="A23" s="6" t="s">
         <v>21</v>
       </c>
@@ -2214,7 +2214,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="24" spans="1:2" ht="60" customHeight="1">
+    <row r="24" spans="1:2" ht="32" customHeight="1">
       <c r="A24" s="6" t="s">
         <v>22</v>
       </c>
@@ -2222,7 +2222,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="25" spans="1:2" ht="46" customHeight="1">
+    <row r="25" spans="1:2" ht="32" customHeight="1">
       <c r="A25" s="6" t="s">
         <v>23</v>
       </c>
@@ -2246,7 +2246,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="28" spans="1:2" ht="46" customHeight="1">
+    <row r="28" spans="1:2" ht="60" customHeight="1">
       <c r="A28" s="6" t="s">
         <v>26</v>
       </c>
@@ -2262,7 +2262,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="30" spans="1:2" ht="60" customHeight="1">
+    <row r="30" spans="1:2" ht="74" customHeight="1">
       <c r="A30" s="6" t="s">
         <v>28</v>
       </c>
@@ -2270,7 +2270,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="31" spans="1:2" ht="32" customHeight="1">
+    <row r="31" spans="1:2" ht="46" customHeight="1">
       <c r="A31" s="6" t="s">
         <v>29</v>
       </c>
@@ -2278,7 +2278,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="32" spans="1:2" ht="32" customHeight="1">
+    <row r="32" spans="1:2" ht="46" customHeight="1">
       <c r="A32" s="6" t="s">
         <v>30</v>
       </c>
@@ -2286,7 +2286,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="33" spans="1:2" ht="46" customHeight="1">
+    <row r="33" spans="1:2" ht="60" customHeight="1">
       <c r="A33" s="6" t="s">
         <v>31</v>
       </c>
@@ -2294,7 +2294,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="34" spans="1:2" ht="46" customHeight="1">
+    <row r="34" spans="1:2" ht="60" customHeight="1">
       <c r="A34" s="6" t="s">
         <v>32</v>
       </c>
@@ -2302,7 +2302,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="35" spans="1:2" ht="60" customHeight="1">
+    <row r="35" spans="1:2" ht="18" customHeight="1">
       <c r="A35" s="6" t="s">
         <v>33</v>
       </c>
@@ -2310,7 +2310,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="36" spans="1:2" ht="46" customHeight="1">
+    <row r="36" spans="1:2" ht="32" customHeight="1">
       <c r="A36" s="6" t="s">
         <v>34</v>
       </c>
@@ -2318,7 +2318,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="37" spans="1:2" ht="60" customHeight="1">
+    <row r="37" spans="1:2" ht="74" customHeight="1">
       <c r="A37" s="6" t="s">
         <v>35</v>
       </c>
@@ -2334,7 +2334,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="39" spans="1:2" ht="46" customHeight="1">
+    <row r="39" spans="1:2" ht="18" customHeight="1">
       <c r="A39" s="6" t="s">
         <v>37</v>
       </c>
@@ -2342,7 +2342,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="40" spans="1:2" ht="60" customHeight="1">
+    <row r="40" spans="1:2" ht="18" customHeight="1">
       <c r="A40" s="6" t="s">
         <v>38</v>
       </c>
@@ -2350,7 +2350,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="41" spans="1:2" ht="60" customHeight="1">
+    <row r="41" spans="1:2" ht="32" customHeight="1">
       <c r="A41" s="6" t="s">
         <v>39</v>
       </c>
@@ -2358,7 +2358,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="42" spans="1:2" ht="18" customHeight="1">
+    <row r="42" spans="1:2" ht="46" customHeight="1">
       <c r="A42" s="6" t="s">
         <v>40</v>
       </c>
@@ -2374,7 +2374,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="44" spans="1:2" ht="74" customHeight="1">
+    <row r="44" spans="1:2" ht="60" customHeight="1">
       <c r="A44" s="6" t="s">
         <v>42</v>
       </c>
@@ -2390,7 +2390,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="46" spans="1:2" ht="18" customHeight="1">
+    <row r="46" spans="1:2" ht="46" customHeight="1">
       <c r="A46" s="6" t="s">
         <v>44</v>
       </c>
@@ -2398,7 +2398,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="47" spans="1:2" ht="18" customHeight="1">
+    <row r="47" spans="1:2" ht="46" customHeight="1">
       <c r="A47" s="6" t="s">
         <v>45</v>
       </c>
@@ -2406,7 +2406,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="48" spans="1:2" ht="32" customHeight="1">
+    <row r="48" spans="1:2" ht="46" customHeight="1">
       <c r="A48" s="6" t="s">
         <v>46</v>
       </c>
@@ -2416,8 +2416,8 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B46" r:id="rId1"/>
-    <hyperlink ref="B47" r:id="rId2"/>
+    <hyperlink ref="B39" r:id="rId1"/>
+    <hyperlink ref="B40" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>